<commit_message>
Auto-generate Excel report from workflow
</commit_message>
<xml_diff>
--- a/data_comp.xlsx
+++ b/data_comp.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,7 +516,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SELECT COUNT(*) FROM DBT_POC.DBT_SCHEMA.FACT_ORDERS WHERE FACT_ORDERS.ORDER_STATUS = 'Completed';</t>
+          <t>SELECT COUNT(*) FROM DBT_POC.DBT_SCHEMA.FACT_ORDERS WHERE ORDER_STATUS = 'Completed';</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -577,26 +577,49 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>SELECT SUM(FACT_ORDER_ITEMS.UNIT_PRICE * FACT_ORDER_ITEMS.QUANTITY) - SUM(FACT_ORDER_ITEMS.DISCOUNT_AMOUNT) FROM FACT_ORDER_ITEMS;</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SELECT SUM(DAILY_REVENUE.DAILY_REV) FROM DAILY_REVENUE;</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>000904 (42000): SQL compilation error: error line 1 at position 11
+invalid identifier 'DAILY_REVENUE.DAILY_REV'</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SELECT DIM_CUSTOMER.CUSTOMER_KEY, DIM_CUSTOMER.CUSTOMER_ID, DIM_CUSTOMER.CUSTOMER_NAME, DIM_CUSTOMER.SEGMENT, DIM_GEOGRAPHY.CITY, DIM_GEOGRAPHY.STATE_REGION, DIM_GEOGRAPHY.COUNTRY FROM DIM_CUSTOMER INNER JOIN DIM_GEOGRAPHY ON DIM_CUSTOMER.GEO_KEY = DIM_GEOGRAPHY.GEO_KEY;</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>-- INVALID SQL
--- Execution failed on sql 'SELECT SUM(FACT_ORDER_ITEMS.UNIT_PRICE * FACT_ORDER_ITEMS.QUANTITY) AS DAILY_REVENUE FROM FACT_ORDER_ITEMS INNER JOIN FACT_ORDERS ON FACT_ORDER_ITEMS.ORDER_ID = FACT_ORDERS.ORDER_ID WHERE FACT_ORDERS.ORDER_DATE_KEY = DAILY_REVENUE.DATE_VALUE;': 000904 (42000): SQL compilation error: error line 1 at position 217
-invalid identifier 'DAILY_REVENUE.DATE_VALUE'
-SELECT SUM(FACT_ORDER_ITEMS.UNIT_PRICE * FACT_ORDER_ITEMS.QUANTITY) AS DAILY_REVENUE FROM FACT_ORDER_ITEMS INNER JOIN FACT_ORDERS ON FACT_ORDER_ITEMS.ORDER_ID = FACT_ORDERS.ORDER_ID WHERE FACT_ORDERS.ORDER_DATE_KEY = DAILY_REVENUE.DATE_VALUE;</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>SELECT SUM(DAILY_REVENUE.DAILY_REVENUE) FROM DAILY_REVENUE;</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+-- Execution failed on sql 'SELECT COUNT(*) FROM DBT_POC.DBT_SCHEMA.DIM_CUSTOMER_ENR;': 002003 (42S02): SQL compilation error:
+Object 'DBT_POC.DBT_SCHEMA.DIM_CUSTOMER_ENR' does not exist or not authorized.
+SELECT COUNT(*) FROM DBT_POC.DBT_SCHEMA.DIM_CUSTOMER_ENR;</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>001003 (42000): SQL compilation error:
-syntax error line 1 at position 0 unexpected 'invalid'.</t>
+syntax error line 1 at position 0 unexpected 'Object'.</t>
         </is>
       </c>
     </row>

</xml_diff>